<commit_message>
test(xlsx): normalize regression fixture structure
</commit_message>
<xml_diff>
--- a/test-data/fixtures/parser-regression/Turnos_Sebastian_Pozo_Mendoza_prueba_cambios.xlsx
+++ b/test-data/fixtures/parser-regression/Turnos_Sebastian_Pozo_Mendoza_prueba_cambios.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="73">
   <si>
     <t>Copia no Controlada si se Imprime - Calendario empleado</t>
   </si>
@@ -298,22 +298,6 @@
   <si>
     <t>Todos los días
 Color</t>
-  </si>
-  <si>
-    <t>20:00 
-04:00</t>
-  </si>
-  <si>
-    <t>06:00 
-14:00</t>
-  </si>
-  <si>
-    <t>18:00 
-02:00</t>
-  </si>
-  <si>
-    <t>16:00 
-00:00</t>
   </si>
 </sst>
 </file>
@@ -922,8 +906,9 @@
       <c r="D4" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="16" t="s">
-        <v>73</v>
+      <c r="E4" s="16" t="str">
+        <v>20:00 
+04:00</v>
       </c>
       <c r="F4" s="17" t="s">
         <v>7</v>
@@ -955,8 +940,9 @@
       <c r="O4" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="P4" s="15" t="s">
-        <v>74</v>
+      <c r="P4" s="15" t="str">
+        <v>06:00 
+14:00</v>
       </c>
       <c r="Q4" s="15" t="s">
         <v>14</v>
@@ -1047,8 +1033,9 @@
       <c r="M5" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="N5" s="15" t="s">
-        <v>75</v>
+      <c r="N5" s="15" t="str">
+        <v>18:00 
+02:00</v>
       </c>
       <c r="O5" s="15" t="s">
         <v>22</v>
@@ -1356,8 +1343,9 @@
       <c r="V8" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="W8" s="15" t="s">
-        <v>76</v>
+      <c r="W8" s="15" t="str">
+        <v>16:00 
+00:00</v>
       </c>
       <c r="X8" s="15" t="s">
         <v>6</v>
@@ -1712,8 +1700,9 @@
       <c r="K12" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="L12" s="15" t="s">
-        <v>74</v>
+      <c r="L12" s="15" t="str">
+        <v>06:00 
+14:00</v>
       </c>
       <c r="M12" s="15" t="s">
         <v>13</v>

</xml_diff>